<commit_message>
chore: checkpoint current project updates
</commit_message>
<xml_diff>
--- a/docs/iFare_問題追蹤與AI維運規劃.xlsx
+++ b/docs/iFare_問題追蹤與AI維運規劃.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A2AE635-A91A-465F-A1F5-145F8E89E0C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{960D9A36-E2A1-4874-8B2A-EBD1CCD90D8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PoC研究" sheetId="1" r:id="rId1"/>
@@ -8523,7 +8523,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P33"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="6" customWidth="1"/>
     <col min="3" max="4" width="17.6640625" customWidth="1"/>
@@ -9360,7 +9360,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>16</v>
       </c>
@@ -9410,7 +9410,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -9460,7 +9460,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>18</v>
       </c>
@@ -9510,7 +9510,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>19</v>
       </c>
@@ -9560,7 +9560,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>20</v>
       </c>
@@ -9610,7 +9610,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>21</v>
       </c>
@@ -9660,7 +9660,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>22</v>
       </c>
@@ -9710,7 +9710,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>23</v>
       </c>
@@ -9760,7 +9760,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>24</v>
       </c>
@@ -9810,7 +9810,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>25</v>
       </c>
@@ -9860,7 +9860,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>26</v>
       </c>
@@ -9910,7 +9910,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="29" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>27</v>
       </c>
@@ -9960,7 +9960,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>28</v>
       </c>
@@ -10010,7 +10010,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>29</v>
       </c>
@@ -10060,7 +10060,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>30</v>
       </c>
@@ -10110,7 +10110,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
         <v>31</v>
       </c>
@@ -10175,7 +10175,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Q127"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="6" customWidth="1"/>
     <col min="3" max="3" width="22.6640625" customWidth="1"/>
@@ -16246,7 +16246,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="117" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A117" s="2">
         <v>114</v>
       </c>
@@ -16299,7 +16299,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="118" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A118" s="2">
         <v>115</v>
       </c>
@@ -16352,7 +16352,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="119" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A119" s="2">
         <v>116</v>
       </c>
@@ -16405,7 +16405,7 @@
         <v>970</v>
       </c>
     </row>
-    <row r="120" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A120" s="2">
         <v>117</v>
       </c>
@@ -16458,7 +16458,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="121" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A121" s="2">
         <v>118</v>
       </c>
@@ -16511,7 +16511,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="122" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A122" s="2">
         <v>119</v>
       </c>
@@ -16564,7 +16564,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="123" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A123" s="2">
         <v>120</v>
       </c>
@@ -16617,7 +16617,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="124" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A124" s="2">
         <v>121</v>
       </c>
@@ -16670,7 +16670,7 @@
         <v>970</v>
       </c>
     </row>
-    <row r="125" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A125" s="2">
         <v>122</v>
       </c>
@@ -16723,7 +16723,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="126" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A126" s="3">
         <v>123</v>
       </c>
@@ -16776,7 +16776,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="127" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A127" s="3">
         <v>124</v>
       </c>
@@ -16844,7 +16844,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P184"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="5.77734375" customWidth="1"/>
     <col min="3" max="3" width="16.109375" customWidth="1"/>
@@ -16862,7 +16862,7 @@
     <col min="16" max="16" width="255.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>1250</v>
       </c>
@@ -16882,7 +16882,7 @@
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
     </row>
-    <row r="2" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -16932,7 +16932,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -16982,7 +16982,7 @@
         <v>1259</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -17032,7 +17032,7 @@
         <v>1265</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -17082,7 +17082,7 @@
         <v>1270</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -17132,7 +17132,7 @@
         <v>1277</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -17182,7 +17182,7 @@
         <v>1281</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -17232,7 +17232,7 @@
         <v>1288</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -17282,7 +17282,7 @@
         <v>1294</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>8</v>
       </c>
@@ -17332,7 +17332,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -17382,7 +17382,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -17432,7 +17432,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -17482,7 +17482,7 @@
         <v>1316</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>12</v>
       </c>
@@ -17532,7 +17532,7 @@
         <v>1322</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -17582,7 +17582,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>14</v>
       </c>
@@ -17632,7 +17632,7 @@
         <v>1335</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>15</v>
       </c>
@@ -17682,7 +17682,7 @@
         <v>1343</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>16</v>
       </c>
@@ -17732,7 +17732,7 @@
         <v>1351</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -17782,7 +17782,7 @@
         <v>1358</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>18</v>
       </c>
@@ -17832,7 +17832,7 @@
         <v>1365</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>19</v>
       </c>
@@ -17882,7 +17882,7 @@
         <v>1370</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>20</v>
       </c>
@@ -17932,7 +17932,7 @@
         <v>1376</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>21</v>
       </c>
@@ -17982,7 +17982,7 @@
         <v>1382</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>22</v>
       </c>
@@ -18032,7 +18032,7 @@
         <v>1390</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>23</v>
       </c>
@@ -18082,7 +18082,7 @@
         <v>1396</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>24</v>
       </c>
@@ -18132,7 +18132,7 @@
         <v>1401</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>25</v>
       </c>
@@ -18182,7 +18182,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>26</v>
       </c>
@@ -18232,7 +18232,7 @@
         <v>1408</v>
       </c>
     </row>
-    <row r="29" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>27</v>
       </c>
@@ -18282,7 +18282,7 @@
         <v>1416</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>28</v>
       </c>
@@ -18332,7 +18332,7 @@
         <v>1422</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>29</v>
       </c>
@@ -18382,7 +18382,7 @@
         <v>1427</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>30</v>
       </c>
@@ -18432,7 +18432,7 @@
         <v>1432</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>31</v>
       </c>
@@ -18482,7 +18482,7 @@
         <v>1436</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>32</v>
       </c>
@@ -18532,7 +18532,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>33</v>
       </c>
@@ -18582,7 +18582,7 @@
         <v>1448</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>34</v>
       </c>
@@ -18632,7 +18632,7 @@
         <v>1453</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
         <v>35</v>
       </c>
@@ -18682,7 +18682,7 @@
         <v>1460</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>36</v>
       </c>
@@ -18732,7 +18732,7 @@
         <v>1468</v>
       </c>
     </row>
-    <row r="39" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
         <v>37</v>
       </c>
@@ -18782,7 +18782,7 @@
         <v>1474</v>
       </c>
     </row>
-    <row r="40" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>38</v>
       </c>
@@ -18832,7 +18832,7 @@
         <v>1479</v>
       </c>
     </row>
-    <row r="41" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>39</v>
       </c>
@@ -18882,7 +18882,7 @@
         <v>1483</v>
       </c>
     </row>
-    <row r="42" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>40</v>
       </c>
@@ -18932,7 +18932,7 @@
         <v>1491</v>
       </c>
     </row>
-    <row r="43" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>41</v>
       </c>
@@ -18982,7 +18982,7 @@
         <v>1498</v>
       </c>
     </row>
-    <row r="44" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <v>42</v>
       </c>
@@ -19032,7 +19032,7 @@
         <v>1504</v>
       </c>
     </row>
-    <row r="45" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
         <v>43</v>
       </c>
@@ -19082,7 +19082,7 @@
         <v>1508</v>
       </c>
     </row>
-    <row r="46" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <v>44</v>
       </c>
@@ -19132,7 +19132,7 @@
         <v>1514</v>
       </c>
     </row>
-    <row r="47" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>45</v>
       </c>
@@ -19182,7 +19182,7 @@
         <v>1519</v>
       </c>
     </row>
-    <row r="48" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>46</v>
       </c>
@@ -19232,7 +19232,7 @@
         <v>1524</v>
       </c>
     </row>
-    <row r="49" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
         <v>47</v>
       </c>
@@ -19282,7 +19282,7 @@
         <v>1530</v>
       </c>
     </row>
-    <row r="50" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
         <v>48</v>
       </c>
@@ -19332,7 +19332,7 @@
         <v>1535</v>
       </c>
     </row>
-    <row r="51" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>49</v>
       </c>
@@ -19382,7 +19382,7 @@
         <v>1541</v>
       </c>
     </row>
-    <row r="52" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
         <v>50</v>
       </c>
@@ -19432,7 +19432,7 @@
         <v>1548</v>
       </c>
     </row>
-    <row r="53" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <v>51</v>
       </c>
@@ -19482,7 +19482,7 @@
         <v>1555</v>
       </c>
     </row>
-    <row r="54" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
         <v>52</v>
       </c>
@@ -19532,7 +19532,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="55" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
         <v>53</v>
       </c>
@@ -19582,7 +19582,7 @@
         <v>1567</v>
       </c>
     </row>
-    <row r="56" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>54</v>
       </c>
@@ -19632,7 +19632,7 @@
         <v>1575</v>
       </c>
     </row>
-    <row r="57" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
         <v>55</v>
       </c>
@@ -19682,7 +19682,7 @@
         <v>1582</v>
       </c>
     </row>
-    <row r="58" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
         <v>56</v>
       </c>
@@ -19732,7 +19732,7 @@
         <v>1587</v>
       </c>
     </row>
-    <row r="59" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
         <v>57</v>
       </c>
@@ -19782,7 +19782,7 @@
         <v>1593</v>
       </c>
     </row>
-    <row r="60" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
         <v>58</v>
       </c>
@@ -19832,7 +19832,7 @@
         <v>1599</v>
       </c>
     </row>
-    <row r="61" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
         <v>59</v>
       </c>
@@ -19882,7 +19882,7 @@
         <v>1606</v>
       </c>
     </row>
-    <row r="62" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
         <v>60</v>
       </c>
@@ -19932,7 +19932,7 @@
         <v>1611</v>
       </c>
     </row>
-    <row r="63" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
         <v>61</v>
       </c>
@@ -19982,7 +19982,7 @@
         <v>1616</v>
       </c>
     </row>
-    <row r="64" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
         <v>62</v>
       </c>
@@ -20032,7 +20032,7 @@
         <v>1621</v>
       </c>
     </row>
-    <row r="65" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
         <v>63</v>
       </c>
@@ -20082,7 +20082,7 @@
         <v>1626</v>
       </c>
     </row>
-    <row r="66" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
         <v>64</v>
       </c>
@@ -20132,7 +20132,7 @@
         <v>1633</v>
       </c>
     </row>
-    <row r="67" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>65</v>
       </c>
@@ -20182,7 +20182,7 @@
         <v>1639</v>
       </c>
     </row>
-    <row r="68" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
         <v>66</v>
       </c>
@@ -20232,7 +20232,7 @@
         <v>1646</v>
       </c>
     </row>
-    <row r="69" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
         <v>67</v>
       </c>
@@ -20282,7 +20282,7 @@
         <v>1651</v>
       </c>
     </row>
-    <row r="70" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
         <v>68</v>
       </c>
@@ -20332,7 +20332,7 @@
         <v>1656</v>
       </c>
     </row>
-    <row r="71" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
         <v>69</v>
       </c>
@@ -20382,7 +20382,7 @@
         <v>1664</v>
       </c>
     </row>
-    <row r="72" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A72" s="2">
         <v>70</v>
       </c>
@@ -20432,7 +20432,7 @@
         <v>1669</v>
       </c>
     </row>
-    <row r="73" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
         <v>71</v>
       </c>
@@ -20482,7 +20482,7 @@
         <v>1675</v>
       </c>
     </row>
-    <row r="74" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A74" s="2">
         <v>72</v>
       </c>
@@ -20532,7 +20532,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="75" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
         <v>73</v>
       </c>
@@ -20582,7 +20582,7 @@
         <v>1687</v>
       </c>
     </row>
-    <row r="76" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
         <v>74</v>
       </c>
@@ -20632,7 +20632,7 @@
         <v>1693</v>
       </c>
     </row>
-    <row r="77" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A77" s="2">
         <v>75</v>
       </c>
@@ -20682,7 +20682,7 @@
         <v>1699</v>
       </c>
     </row>
-    <row r="78" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A78" s="2">
         <v>76</v>
       </c>
@@ -20732,7 +20732,7 @@
         <v>1705</v>
       </c>
     </row>
-    <row r="79" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
         <v>77</v>
       </c>
@@ -20782,7 +20782,7 @@
         <v>1711</v>
       </c>
     </row>
-    <row r="80" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
         <v>78</v>
       </c>
@@ -20832,7 +20832,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="81" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
         <v>79</v>
       </c>
@@ -20882,7 +20882,7 @@
         <v>1723</v>
       </c>
     </row>
-    <row r="82" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
         <v>80</v>
       </c>
@@ -20932,7 +20932,7 @@
         <v>1729</v>
       </c>
     </row>
-    <row r="83" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
         <v>81</v>
       </c>
@@ -20982,7 +20982,7 @@
         <v>1736</v>
       </c>
     </row>
-    <row r="84" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A84" s="2">
         <v>82</v>
       </c>
@@ -21032,7 +21032,7 @@
         <v>1743</v>
       </c>
     </row>
-    <row r="85" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A85" s="2">
         <v>83</v>
       </c>
@@ -21082,7 +21082,7 @@
         <v>1749</v>
       </c>
     </row>
-    <row r="86" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A86" s="2">
         <v>84</v>
       </c>
@@ -21132,7 +21132,7 @@
         <v>1755</v>
       </c>
     </row>
-    <row r="87" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A87" s="2">
         <v>85</v>
       </c>
@@ -21182,7 +21182,7 @@
         <v>1761</v>
       </c>
     </row>
-    <row r="88" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A88" s="2">
         <v>86</v>
       </c>
@@ -21232,7 +21232,7 @@
         <v>1769</v>
       </c>
     </row>
-    <row r="89" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A89" s="2">
         <v>87</v>
       </c>
@@ -21282,7 +21282,7 @@
         <v>1775</v>
       </c>
     </row>
-    <row r="90" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A90" s="2">
         <v>88</v>
       </c>
@@ -21332,7 +21332,7 @@
         <v>1781</v>
       </c>
     </row>
-    <row r="91" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A91" s="2">
         <v>89</v>
       </c>
@@ -21382,7 +21382,7 @@
         <v>1786</v>
       </c>
     </row>
-    <row r="92" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A92" s="2">
         <v>90</v>
       </c>
@@ -21432,7 +21432,7 @@
         <v>1786</v>
       </c>
     </row>
-    <row r="93" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A93" s="2">
         <v>91</v>
       </c>
@@ -21482,7 +21482,7 @@
         <v>1786</v>
       </c>
     </row>
-    <row r="94" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A94" s="2">
         <v>92</v>
       </c>
@@ -21532,7 +21532,7 @@
         <v>1802</v>
       </c>
     </row>
-    <row r="95" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A95" s="2">
         <v>93</v>
       </c>
@@ -21582,7 +21582,7 @@
         <v>1808</v>
       </c>
     </row>
-    <row r="96" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A96" s="2">
         <v>94</v>
       </c>
@@ -21632,7 +21632,7 @@
         <v>1786</v>
       </c>
     </row>
-    <row r="97" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A97" s="2">
         <v>95</v>
       </c>
@@ -21682,7 +21682,7 @@
         <v>1786</v>
       </c>
     </row>
-    <row r="98" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A98" s="2">
         <v>96</v>
       </c>
@@ -21732,7 +21732,7 @@
         <v>1823</v>
       </c>
     </row>
-    <row r="99" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A99" s="2">
         <v>97</v>
       </c>
@@ -21782,7 +21782,7 @@
         <v>1786</v>
       </c>
     </row>
-    <row r="100" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A100" s="2">
         <v>98</v>
       </c>
@@ -21832,7 +21832,7 @@
         <v>1836</v>
       </c>
     </row>
-    <row r="101" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A101" s="2">
         <v>99</v>
       </c>
@@ -21882,7 +21882,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="102" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A102" s="2">
         <v>100</v>
       </c>
@@ -21932,7 +21932,7 @@
         <v>1849</v>
       </c>
     </row>
-    <row r="103" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A103" s="2">
         <v>101</v>
       </c>
@@ -21982,7 +21982,7 @@
         <v>1856</v>
       </c>
     </row>
-    <row r="104" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A104" s="2">
         <v>102</v>
       </c>
@@ -22032,7 +22032,7 @@
         <v>1864</v>
       </c>
     </row>
-    <row r="105" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A105" s="2">
         <v>103</v>
       </c>
@@ -22082,7 +22082,7 @@
         <v>1871</v>
       </c>
     </row>
-    <row r="106" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A106" s="2">
         <v>104</v>
       </c>
@@ -22132,7 +22132,7 @@
         <v>1878</v>
       </c>
     </row>
-    <row r="107" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A107" s="2">
         <v>105</v>
       </c>
@@ -22182,7 +22182,7 @@
         <v>1885</v>
       </c>
     </row>
-    <row r="108" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A108" s="2">
         <v>106</v>
       </c>
@@ -22232,7 +22232,7 @@
         <v>1894</v>
       </c>
     </row>
-    <row r="109" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A109" s="2">
         <v>107</v>
       </c>
@@ -22282,7 +22282,7 @@
         <v>1902</v>
       </c>
     </row>
-    <row r="110" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A110" s="2">
         <v>108</v>
       </c>
@@ -22332,7 +22332,7 @@
         <v>1909</v>
       </c>
     </row>
-    <row r="111" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A111" s="2">
         <v>109</v>
       </c>
@@ -22382,7 +22382,7 @@
         <v>1916</v>
       </c>
     </row>
-    <row r="112" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A112" s="2">
         <v>110</v>
       </c>
@@ -22432,7 +22432,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="113" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A113" s="2">
         <v>111</v>
       </c>
@@ -22482,7 +22482,7 @@
         <v>1933</v>
       </c>
     </row>
-    <row r="114" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A114" s="2">
         <v>112</v>
       </c>
@@ -22532,7 +22532,7 @@
         <v>1941</v>
       </c>
     </row>
-    <row r="115" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A115" s="2">
         <v>113</v>
       </c>
@@ -22582,7 +22582,7 @@
         <v>1949</v>
       </c>
     </row>
-    <row r="116" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A116" s="2">
         <v>114</v>
       </c>
@@ -22632,7 +22632,7 @@
         <v>1957</v>
       </c>
     </row>
-    <row r="117" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A117" s="2">
         <v>115</v>
       </c>
@@ -22682,7 +22682,7 @@
         <v>1965</v>
       </c>
     </row>
-    <row r="118" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A118" s="2">
         <v>116</v>
       </c>
@@ -22732,7 +22732,7 @@
         <v>1973</v>
       </c>
     </row>
-    <row r="119" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A119" s="2">
         <v>117</v>
       </c>
@@ -22782,7 +22782,7 @@
         <v>1980</v>
       </c>
     </row>
-    <row r="120" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A120" s="2">
         <v>118</v>
       </c>
@@ -22832,7 +22832,7 @@
         <v>1988</v>
       </c>
     </row>
-    <row r="121" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A121" s="2">
         <v>119</v>
       </c>
@@ -22882,7 +22882,7 @@
         <v>1997</v>
       </c>
     </row>
-    <row r="122" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A122" s="2">
         <v>120</v>
       </c>
@@ -22932,7 +22932,7 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="123" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A123" s="2">
         <v>121</v>
       </c>
@@ -22982,7 +22982,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="124" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A124" s="2">
         <v>122</v>
       </c>
@@ -23032,7 +23032,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="125" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A125" s="2">
         <v>123</v>
       </c>
@@ -23082,7 +23082,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="126" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A126" s="2">
         <v>124</v>
       </c>
@@ -23132,7 +23132,7 @@
         <v>2033</v>
       </c>
     </row>
-    <row r="127" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A127" s="2">
         <v>125</v>
       </c>
@@ -23182,7 +23182,7 @@
         <v>2040</v>
       </c>
     </row>
-    <row r="128" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A128" s="2">
         <v>126</v>
       </c>
@@ -23232,7 +23232,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="129" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A129" s="2">
         <v>127</v>
       </c>
@@ -23282,7 +23282,7 @@
         <v>2056</v>
       </c>
     </row>
-    <row r="130" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A130" s="2">
         <v>128</v>
       </c>
@@ -23332,7 +23332,7 @@
         <v>2065</v>
       </c>
     </row>
-    <row r="131" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A131" s="2">
         <v>129</v>
       </c>
@@ -23382,7 +23382,7 @@
         <v>2073</v>
       </c>
     </row>
-    <row r="132" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A132" s="2">
         <v>130</v>
       </c>
@@ -23432,7 +23432,7 @@
         <v>2079</v>
       </c>
     </row>
-    <row r="133" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A133" s="2">
         <v>131</v>
       </c>
@@ -23482,7 +23482,7 @@
         <v>2088</v>
       </c>
     </row>
-    <row r="134" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A134" s="2">
         <v>132</v>
       </c>
@@ -23532,7 +23532,7 @@
         <v>2095</v>
       </c>
     </row>
-    <row r="135" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A135" s="2">
         <v>133</v>
       </c>
@@ -23582,7 +23582,7 @@
         <v>2103</v>
       </c>
     </row>
-    <row r="136" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A136" s="2">
         <v>134</v>
       </c>
@@ -23632,7 +23632,7 @@
         <v>2110</v>
       </c>
     </row>
-    <row r="137" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A137" s="2">
         <v>135</v>
       </c>
@@ -23682,7 +23682,7 @@
         <v>2117</v>
       </c>
     </row>
-    <row r="138" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A138" s="2">
         <v>136</v>
       </c>
@@ -23732,7 +23732,7 @@
         <v>2124</v>
       </c>
     </row>
-    <row r="139" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A139" s="2">
         <v>137</v>
       </c>
@@ -23782,7 +23782,7 @@
         <v>2130</v>
       </c>
     </row>
-    <row r="140" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A140" s="2">
         <v>138</v>
       </c>
@@ -23832,7 +23832,7 @@
         <v>2136</v>
       </c>
     </row>
-    <row r="141" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A141" s="2">
         <v>139</v>
       </c>
@@ -23882,7 +23882,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="142" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A142" s="2">
         <v>140</v>
       </c>
@@ -23932,7 +23932,7 @@
         <v>2148</v>
       </c>
     </row>
-    <row r="143" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A143" s="2">
         <v>141</v>
       </c>
@@ -23982,7 +23982,7 @@
         <v>2155</v>
       </c>
     </row>
-    <row r="144" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A144" s="2">
         <v>142</v>
       </c>
@@ -24032,7 +24032,7 @@
         <v>2162</v>
       </c>
     </row>
-    <row r="145" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A145" s="2">
         <v>143</v>
       </c>
@@ -24082,7 +24082,7 @@
         <v>2171</v>
       </c>
     </row>
-    <row r="146" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A146" s="2">
         <v>144</v>
       </c>
@@ -24132,7 +24132,7 @@
         <v>2179</v>
       </c>
     </row>
-    <row r="147" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A147" s="2">
         <v>145</v>
       </c>
@@ -24182,7 +24182,7 @@
         <v>2188</v>
       </c>
     </row>
-    <row r="148" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A148" s="2">
         <v>146</v>
       </c>
@@ -24232,7 +24232,7 @@
         <v>2195</v>
       </c>
     </row>
-    <row r="149" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A149" s="2">
         <v>147</v>
       </c>
@@ -24282,7 +24282,7 @@
         <v>2203</v>
       </c>
     </row>
-    <row r="150" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A150" s="2">
         <v>148</v>
       </c>
@@ -24332,7 +24332,7 @@
         <v>2211</v>
       </c>
     </row>
-    <row r="151" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A151" s="2">
         <v>149</v>
       </c>
@@ -24382,7 +24382,7 @@
         <v>2219</v>
       </c>
     </row>
-    <row r="152" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A152" s="2">
         <v>150</v>
       </c>
@@ -24432,7 +24432,7 @@
         <v>2228</v>
       </c>
     </row>
-    <row r="153" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A153" s="2">
         <v>151</v>
       </c>
@@ -24482,7 +24482,7 @@
         <v>2237</v>
       </c>
     </row>
-    <row r="154" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A154" s="2">
         <v>152</v>
       </c>
@@ -24532,7 +24532,7 @@
         <v>2244</v>
       </c>
     </row>
-    <row r="155" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A155" s="2">
         <v>153</v>
       </c>
@@ -24582,7 +24582,7 @@
         <v>2252</v>
       </c>
     </row>
-    <row r="156" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A156" s="2">
         <v>154</v>
       </c>
@@ -24632,7 +24632,7 @@
         <v>2260</v>
       </c>
     </row>
-    <row r="157" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A157" s="2">
         <v>155</v>
       </c>
@@ -24682,7 +24682,7 @@
         <v>2267</v>
       </c>
     </row>
-    <row r="158" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A158" s="2">
         <v>156</v>
       </c>
@@ -24732,7 +24732,7 @@
         <v>2275</v>
       </c>
     </row>
-    <row r="159" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A159" s="2">
         <v>157</v>
       </c>
@@ -24782,7 +24782,7 @@
         <v>2283</v>
       </c>
     </row>
-    <row r="160" spans="1:16" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A160" s="2">
         <v>158</v>
       </c>
@@ -24832,7 +24832,7 @@
         <v>2291</v>
       </c>
     </row>
-    <row r="161" spans="1:16" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A161" s="2">
         <v>159</v>
       </c>
@@ -24882,7 +24882,7 @@
         <v>2299</v>
       </c>
     </row>
-    <row r="162" spans="1:16" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A162" s="2">
         <v>160</v>
       </c>
@@ -24932,7 +24932,7 @@
         <v>2305</v>
       </c>
     </row>
-    <row r="163" spans="1:16" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A163" s="2">
         <v>161</v>
       </c>
@@ -24982,7 +24982,7 @@
         <v>2313</v>
       </c>
     </row>
-    <row r="164" spans="1:16" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A164" s="2">
         <v>162</v>
       </c>
@@ -25032,7 +25032,7 @@
         <v>2319</v>
       </c>
     </row>
-    <row r="165" spans="1:16" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A165" s="2">
         <v>163</v>
       </c>
@@ -25082,7 +25082,7 @@
         <v>2327</v>
       </c>
     </row>
-    <row r="166" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A166" s="2">
         <v>164</v>
       </c>
@@ -25132,7 +25132,7 @@
         <v>2334</v>
       </c>
     </row>
-    <row r="167" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A167" s="2">
         <v>165</v>
       </c>
@@ -25182,7 +25182,7 @@
         <v>2341</v>
       </c>
     </row>
-    <row r="168" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A168" s="2">
         <v>166</v>
       </c>
@@ -25232,7 +25232,7 @@
         <v>2349</v>
       </c>
     </row>
-    <row r="169" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A169" s="2">
         <v>167</v>
       </c>
@@ -25282,7 +25282,7 @@
         <v>2356</v>
       </c>
     </row>
-    <row r="170" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A170" s="2">
         <v>168</v>
       </c>
@@ -25332,7 +25332,7 @@
         <v>2365</v>
       </c>
     </row>
-    <row r="171" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A171" s="2">
         <v>169</v>
       </c>
@@ -25382,7 +25382,7 @@
         <v>2372</v>
       </c>
     </row>
-    <row r="172" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A172" s="2">
         <v>170</v>
       </c>
@@ -25432,7 +25432,7 @@
         <v>2379</v>
       </c>
     </row>
-    <row r="173" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A173" s="2">
         <v>171</v>
       </c>
@@ -25482,7 +25482,7 @@
         <v>2387</v>
       </c>
     </row>
-    <row r="174" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A174" s="2">
         <v>172</v>
       </c>
@@ -25532,7 +25532,7 @@
         <v>2394</v>
       </c>
     </row>
-    <row r="175" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A175" s="2">
         <v>173</v>
       </c>
@@ -25582,7 +25582,7 @@
         <v>2402</v>
       </c>
     </row>
-    <row r="176" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A176" s="2">
         <v>174</v>
       </c>
@@ -25632,7 +25632,7 @@
         <v>2409</v>
       </c>
     </row>
-    <row r="177" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A177" s="2">
         <v>175</v>
       </c>
@@ -25682,7 +25682,7 @@
         <v>2418</v>
       </c>
     </row>
-    <row r="178" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A178" s="2">
         <v>176</v>
       </c>
@@ -25732,7 +25732,7 @@
         <v>2427</v>
       </c>
     </row>
-    <row r="179" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A179" s="2">
         <v>177</v>
       </c>
@@ -25782,7 +25782,7 @@
         <v>2437</v>
       </c>
     </row>
-    <row r="180" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A180" s="2">
         <v>178</v>
       </c>
@@ -25832,7 +25832,7 @@
         <v>2445</v>
       </c>
     </row>
-    <row r="181" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A181" s="2">
         <v>179</v>
       </c>
@@ -25882,7 +25882,7 @@
         <v>2454</v>
       </c>
     </row>
-    <row r="182" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A182" s="2">
         <v>180</v>
       </c>
@@ -25932,7 +25932,7 @@
         <v>2463</v>
       </c>
     </row>
-    <row r="183" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A183" s="2">
         <v>181</v>
       </c>
@@ -25982,7 +25982,7 @@
         <v>2472</v>
       </c>
     </row>
-    <row r="184" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A184" s="2">
         <v>182</v>
       </c>
@@ -26047,7 +26047,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H117"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" customWidth="1"/>
     <col min="2" max="2" width="12.5546875" customWidth="1"/>

</xml_diff>